<commit_message>
Add CSV download for calculation history, with tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmNGSmzX2eAZGmmm1twA47
</commit_message>
<xml_diff>
--- a/calculator_test_spec.xlsx
+++ b/calculator_test_spec.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">テスト項目!$1:$1</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">テスト項目!$A$1:$J$70</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">テスト項目!$A$1:$J$75</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="391">
   <si>
     <t xml:space="preserve">電卓アプリ テスト仕様書兼結果表</t>
   </si>
@@ -87,7 +87,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8c22fff </t>
+      <t xml:space="preserve">0e1d16d </t>
     </r>
     <r>
       <rPr>
@@ -158,7 +158,41 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">文字削除、パーセント、履歴、キーボード操作</t>
+      <t xml:space="preserve">文字削除、パーセント、履歴</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(CSV</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ダウンロード含む</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、キーボード操作</t>
     </r>
   </si>
   <si>
@@ -172,7 +206,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Chromium 141(Playwright </t>
+      <t xml:space="preserve">Chromium 141.0.7390.37(Playwright </t>
     </r>
     <r>
       <rPr>
@@ -197,23 +231,6 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Meiryo"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Linux</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">。画面サイズ </t>
     </r>
     <r>
@@ -241,6 +258,23 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">360×640)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。対象</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: file:///home/user/try_claude/index.html</t>
     </r>
   </si>
   <si>
@@ -6925,6 +6959,856 @@
     <t xml:space="preserve">T057</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ダウンロードボタンの状態</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">履歴なし</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">履歴が空の状態で画面を表示する</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">「ダウンロード」ボタンが押せない状態</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">グレー表示</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">になっている</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">履歴なしのとき、ダウンロードボタンの無効状態</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=true</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">履歴のダウンロード</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 + 2 = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を実行し、「ダウンロード」ボタンを押す</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">calculator-history_YYYYMMDD.csv(YYYYMMDD </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">は当日の日付</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">がダウンロードされる。ボタンは押せる状態になっている</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ボタン有効</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、ファイル名「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">calculator-history_20261006.csv</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">」</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T059</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CSV </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の内容</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 + 2 × 3 = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の後、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">のあと </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 ÷ 4 = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を実行し、ダウンロードした</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CSV</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を確認する</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">行目が「日時</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">式</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">結果」。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">行目以降は古い順で「日時</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(YYYY-MM-DD HH:mm:ss),1+2×3,7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">」「日時</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">,8÷4,2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">」の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CSV: ["</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日時</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">式</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">結果</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">","&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日時</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&gt;,1+2×3,7","&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日時</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&gt;,8÷4,2",""]</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T060</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CSV </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の文字コード</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Excel </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で文字化けしない</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ダウンロードした</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CSV</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Excel </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で開く</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ファイルの先頭に </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">UTF-8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BOM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">が付いている</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">見出し</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日時・式・結果</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">や </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×÷ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の記号が文字化けせず表示される</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">先頭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">バイトが </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">UTF-8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BOM(EF BB BF)=true(Excel </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">での目視確認は手動</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">履歴消去後のダウンロードボタン</t>
+  </si>
+  <si>
+    <t xml:space="preserve">履歴がある状態で「履歴を消去」を押す</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「ダウンロード」ボタンが押せない状態に戻る</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">消去前の無効状態</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=false</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、消去後の無効状態</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=true</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T062</t>
+  </si>
+  <si>
     <t xml:space="preserve">キーボード操作</t>
   </si>
   <si>
@@ -7055,7 +7939,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T058</t>
+    <t xml:space="preserve">T063</t>
   </si>
   <si>
     <t xml:space="preserve">演算子キー</t>
@@ -7141,7 +8025,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T059</t>
+    <t xml:space="preserve">T064</t>
   </si>
   <si>
     <t xml:space="preserve">割り算キー</t>
@@ -7306,7 +8190,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T060</t>
+    <t xml:space="preserve">T065</t>
   </si>
   <si>
     <r>
@@ -7382,7 +8266,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T061</t>
+    <t xml:space="preserve">T066</t>
   </si>
   <si>
     <r>
@@ -7439,7 +8323,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T062</t>
+    <t xml:space="preserve">T067</t>
   </si>
   <si>
     <t xml:space="preserve">Backspace</t>
@@ -7481,7 +8365,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T063</t>
+    <t xml:space="preserve">T068</t>
   </si>
   <si>
     <t xml:space="preserve">Esc / Delete</t>
@@ -7610,7 +8494,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T064</t>
+    <t xml:space="preserve">T069</t>
   </si>
   <si>
     <t xml:space="preserve">小数点とパーセント</t>
@@ -7643,7 +8527,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T065</t>
+    <t xml:space="preserve">T070</t>
   </si>
   <si>
     <t xml:space="preserve">動作環境</t>
@@ -7732,7 +8616,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">UA: Chrome/141.0.0.0</t>
+      <t xml:space="preserve">UA: Chrome/141.0.7390.37</t>
     </r>
   </si>
   <si>
@@ -7789,7 +8673,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T066</t>
+    <t xml:space="preserve">T071</t>
   </si>
   <si>
     <t xml:space="preserve">Edge</t>
@@ -7850,7 +8734,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T067</t>
+    <t xml:space="preserve">T072</t>
   </si>
   <si>
     <t xml:space="preserve">Safari / iPhone</t>
@@ -7981,7 +8865,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T068</t>
+    <t xml:space="preserve">T073</t>
   </si>
   <si>
     <t xml:space="preserve">Android Chrome</t>
@@ -8076,7 +8960,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">T069</t>
+    <t xml:space="preserve">T074</t>
   </si>
   <si>
     <t xml:space="preserve">GitHub Pages</t>
@@ -8791,7 +9675,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -8836,8 +9720,8 @@
         <v>16</v>
       </c>
       <c r="B12" s="6" t="n">
-        <f aca="false">COUNTA(テスト項目!A2:A70)</f>
-        <v>69</v>
+        <f aca="false">COUNTA(テスト項目!A2:A75)</f>
+        <v>74</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8845,8 +9729,8 @@
         <v>17</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">COUNTIF(テスト項目!G2:G70,"OK")</f>
-        <v>65</v>
+        <f aca="false">COUNTIF(テスト項目!G2:G75,"OK")</f>
+        <v>70</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8854,7 +9738,7 @@
         <v>18</v>
       </c>
       <c r="B14" s="6" t="n">
-        <f aca="false">COUNTIF(テスト項目!G2:G70,"NG")</f>
+        <f aca="false">COUNTIF(テスト項目!G2:G75,"NG")</f>
         <v>0</v>
       </c>
     </row>
@@ -8873,7 +9757,7 @@
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">IF(B12=0,0,(B13+B14)/B12)</f>
-        <v>0.942028985507246</v>
+        <v>0.945945945945946</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8901,7 +9785,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J75"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -10628,24 +11512,24 @@
       </c>
       <c r="J57" s="12"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
         <v>309</v>
       </c>
       <c r="B58" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C58" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="C58" s="12" t="s">
+      <c r="D58" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="D58" s="12" t="s">
+      <c r="E58" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="E58" s="12" t="s">
+      <c r="F58" s="12" t="s">
         <v>313</v>
-      </c>
-      <c r="F58" s="12" t="s">
-        <v>314</v>
       </c>
       <c r="G58" s="11" t="s">
         <v>17</v>
@@ -10658,24 +11542,24 @@
       </c>
       <c r="J58" s="12"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="B59" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C59" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="B59" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="C59" s="12" t="s">
+      <c r="D59" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="D59" s="12" t="s">
+      <c r="E59" s="13" t="s">
         <v>317</v>
       </c>
-      <c r="E59" s="12" t="s">
+      <c r="F59" s="12" t="s">
         <v>318</v>
-      </c>
-      <c r="F59" s="12" t="s">
-        <v>68</v>
       </c>
       <c r="G59" s="11" t="s">
         <v>17</v>
@@ -10688,23 +11572,23 @@
       </c>
       <c r="J59" s="12"/>
     </row>
-    <row r="60" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="s">
         <v>319</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="C60" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C60" s="13" t="s">
         <v>320</v>
       </c>
-      <c r="D60" s="12" t="s">
+      <c r="D60" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="E60" s="12" t="s">
+      <c r="E60" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="F60" s="12" t="s">
+      <c r="F60" s="13" t="s">
         <v>323</v>
       </c>
       <c r="G60" s="11" t="s">
@@ -10718,14 +11602,14 @@
       </c>
       <c r="J60" s="12"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
         <v>324</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="C61" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C61" s="13" t="s">
         <v>325</v>
       </c>
       <c r="D61" s="12" t="s">
@@ -10735,7 +11619,7 @@
         <v>327</v>
       </c>
       <c r="F61" s="12" t="s">
-        <v>107</v>
+        <v>328</v>
       </c>
       <c r="G61" s="11" t="s">
         <v>17</v>
@@ -10750,22 +11634,22 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>310</v>
+        <v>265</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>57</v>
+        <v>332</v>
       </c>
       <c r="F62" s="12" t="s">
-        <v>58</v>
+        <v>333</v>
       </c>
       <c r="G62" s="11" t="s">
         <v>17</v>
@@ -10780,22 +11664,22 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="C63" s="13" t="s">
-        <v>332</v>
+        <v>335</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>336</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="E63" s="12" t="s">
-        <v>207</v>
+        <v>338</v>
       </c>
       <c r="F63" s="12" t="s">
-        <v>208</v>
+        <v>339</v>
       </c>
       <c r="G63" s="11" t="s">
         <v>17</v>
@@ -10810,22 +11694,22 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="11" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="C64" s="13" t="s">
         <v>335</v>
       </c>
+      <c r="C64" s="12" t="s">
+        <v>341</v>
+      </c>
       <c r="D64" s="12" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="E64" s="12" t="s">
-        <v>221</v>
-      </c>
-      <c r="F64" s="13" t="s">
-        <v>337</v>
+        <v>343</v>
+      </c>
+      <c r="F64" s="12" t="s">
+        <v>68</v>
       </c>
       <c r="G64" s="11" t="s">
         <v>17</v>
@@ -10838,24 +11722,24 @@
       </c>
       <c r="J64" s="12"/>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>310</v>
+        <v>335</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E65" s="12" t="s">
-        <v>238</v>
+        <v>347</v>
       </c>
       <c r="F65" s="12" t="s">
-        <v>127</v>
+        <v>348</v>
       </c>
       <c r="G65" s="11" t="s">
         <v>17</v>
@@ -10868,24 +11752,24 @@
       </c>
       <c r="J65" s="12"/>
     </row>
-    <row r="66" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="C66" s="13" t="s">
-        <v>343</v>
-      </c>
-      <c r="D66" s="13" t="s">
-        <v>344</v>
+        <v>335</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>351</v>
       </c>
       <c r="E66" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="F66" s="13" t="s">
-        <v>346</v>
+        <v>352</v>
+      </c>
+      <c r="F66" s="12" t="s">
+        <v>107</v>
       </c>
       <c r="G66" s="11" t="s">
         <v>17</v>
@@ -10896,117 +11780,267 @@
       <c r="I66" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="J66" s="13" t="s">
-        <v>347</v>
-      </c>
+      <c r="J66" s="12"/>
     </row>
-    <row r="67" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="C67" s="13" t="s">
-        <v>349</v>
-      </c>
-      <c r="D67" s="13" t="s">
-        <v>350</v>
+        <v>335</v>
+      </c>
+      <c r="C67" s="12" t="s">
+        <v>354</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>355</v>
       </c>
       <c r="E67" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="F67" s="12"/>
-      <c r="G67" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F67" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="G67" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H67" s="14" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I67" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="J67" s="12"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="11" t="s">
+        <v>356</v>
+      </c>
+      <c r="B68" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="C68" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>358</v>
+      </c>
+      <c r="E68" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="F68" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="G68" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H68" s="14" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I68" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="J68" s="12"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="B69" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="C69" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>361</v>
+      </c>
+      <c r="E69" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="F69" s="13" t="s">
+        <v>362</v>
+      </c>
+      <c r="G69" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H69" s="14" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I69" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="J69" s="12"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="B70" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="C70" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="D70" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="E70" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="F70" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="G70" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H70" s="14" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I70" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="J70" s="12"/>
+    </row>
+    <row r="71" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="B71" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C71" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="D71" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="E71" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="F71" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="G71" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H71" s="14" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I71" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="J71" s="13" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="11" t="s">
+        <v>373</v>
+      </c>
+      <c r="B72" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C72" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="D72" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="E72" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="F72" s="12"/>
+      <c r="G72" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="H67" s="14"/>
-      <c r="I67" s="12"/>
-      <c r="J67" s="13" t="s">
-        <v>351</v>
+      <c r="H72" s="14"/>
+      <c r="I72" s="12"/>
+      <c r="J72" s="13" t="s">
+        <v>376</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="11" t="s">
-        <v>352</v>
-      </c>
-      <c r="B68" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="C68" s="13" t="s">
-        <v>353</v>
-      </c>
-      <c r="D68" s="13" t="s">
-        <v>354</v>
-      </c>
-      <c r="E68" s="12" t="s">
-        <v>355</v>
-      </c>
-      <c r="F68" s="12"/>
-      <c r="G68" s="15" t="s">
+    <row r="73" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="B73" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C73" s="13" t="s">
+        <v>378</v>
+      </c>
+      <c r="D73" s="13" t="s">
+        <v>379</v>
+      </c>
+      <c r="E73" s="12" t="s">
+        <v>380</v>
+      </c>
+      <c r="F73" s="12"/>
+      <c r="G73" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="H68" s="14"/>
-      <c r="I68" s="12"/>
-      <c r="J68" s="13" t="s">
-        <v>356</v>
+      <c r="H73" s="14"/>
+      <c r="I73" s="12"/>
+      <c r="J73" s="13" t="s">
+        <v>381</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="11" t="s">
-        <v>357</v>
-      </c>
-      <c r="B69" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="C69" s="13" t="s">
-        <v>358</v>
-      </c>
-      <c r="D69" s="13" t="s">
-        <v>359</v>
-      </c>
-      <c r="E69" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="F69" s="12"/>
-      <c r="G69" s="15" t="s">
+    <row r="74" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="11" t="s">
+        <v>382</v>
+      </c>
+      <c r="B74" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C74" s="13" t="s">
+        <v>383</v>
+      </c>
+      <c r="D74" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="E74" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="F74" s="12"/>
+      <c r="G74" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="H69" s="14"/>
-      <c r="I69" s="12"/>
-      <c r="J69" s="13" t="s">
-        <v>360</v>
+      <c r="H74" s="14"/>
+      <c r="I74" s="12"/>
+      <c r="J74" s="13" t="s">
+        <v>385</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="11" t="s">
-        <v>361</v>
-      </c>
-      <c r="B70" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="C70" s="13" t="s">
-        <v>362</v>
-      </c>
-      <c r="D70" s="12" t="s">
-        <v>363</v>
-      </c>
-      <c r="E70" s="12" t="s">
-        <v>364</v>
-      </c>
-      <c r="F70" s="12"/>
-      <c r="G70" s="15" t="s">
+    <row r="75" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="B75" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C75" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="D75" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="E75" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="F75" s="12"/>
+      <c r="G75" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="H70" s="14"/>
-      <c r="I70" s="12"/>
-      <c r="J70" s="12" t="s">
-        <v>365</v>
+      <c r="H75" s="14"/>
+      <c r="I75" s="12"/>
+      <c r="J75" s="12" t="s">
+        <v>390</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J70"/>
-  <conditionalFormatting sqref="G2:G70">
+  <autoFilter ref="A1:J75"/>
+  <conditionalFormatting sqref="G2:G75">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"OK"</formula>
     </cfRule>
@@ -11018,7 +12052,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G70" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G75" type="list">
       <formula1>"OK,NG,未実施"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>